<commit_message>
Petite Cup 53 (S4 Round 3): Lexer finally wins one
Lexer takes it from RoundNzt, with justMaki 3rd and Quickracer10 4th. 29
racers. Maps: PCDJ #52 - Bankbanknewnew by [CSC] Shadynook and PCDJ #52 - A
Little Bit of Bob by [CSC] redal; neither mapper joined the lobby, so nobody is
excluded and all 29 roster entries raced.

This is Lexer's first petite win in the data we hold. Across Seasons 2, 3 and 4
he had no wins at all from four second places and two thirds, never finishing
better than 2nd. We have no Season 1 results, so this is a first within our
records rather than a first outright. He gets the 1st Win badge, which is the
case the milestone fix last week was written for.

No discovery rounds this week (rounds ran 82-84s), so the 14 elimination rounds
map 1:1 onto plugin rounds 8-21. No DNF overrides. Cup strength 88.9% against
COTD 163.

Seasons 2 and 3 are untouched, including their SOF values.
</commit_message>
<xml_diff>
--- a/Petite Cups 51-55.xlsx
+++ b/Petite Cups 51-55.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J59"/>
+  <dimension ref="A2:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -427,6 +427,11 @@
           <t>Petite Cup 52</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Petite Cup 53</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -439,6 +444,11 @@
           <t>Maps: PCDJ - Ridge + Polymer Composite Derivative Junction, by justMaki &amp; agix</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #52 - Bankbanknewnew by [CSC] Shadynook + PCDJ #52 - A Little Bit of Bob by [CSC] redal</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -477,6 +487,26 @@
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -505,6 +535,17 @@
       <c r="I6" t="n">
         <v>23.46221</v>
       </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>22.94841</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -537,6 +578,20 @@
       <c r="J7" t="n">
         <v>13</v>
       </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>22.96622</v>
+      </c>
+      <c r="P7" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -567,6 +622,20 @@
       <c r="J8" t="n">
         <v>12</v>
       </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>23.51184</v>
+      </c>
+      <c r="P8" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -597,6 +666,22 @@
       <c r="J9" t="n">
         <v>11</v>
       </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>[KURK] Quickracer10</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -629,6 +714,20 @@
       <c r="J10" t="n">
         <v>10</v>
       </c>
+      <c r="M10" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Jake</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>23.5223</v>
+      </c>
+      <c r="P10" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -661,6 +760,20 @@
       <c r="J11" t="n">
         <v>9</v>
       </c>
+      <c r="M11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Warsnac</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>23.21611</v>
+      </c>
+      <c r="P11" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -691,6 +804,20 @@
       <c r="J12" t="n">
         <v>8</v>
       </c>
+      <c r="M12" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Azalea</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>23.57596</v>
+      </c>
+      <c r="P12" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -721,6 +848,20 @@
       <c r="J13" t="n">
         <v>8</v>
       </c>
+      <c r="M13" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>[CSC]IronDragon111000</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>23.74276</v>
+      </c>
+      <c r="P13" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -751,6 +892,20 @@
       <c r="J14" t="n">
         <v>7</v>
       </c>
+      <c r="M14" t="n">
+        <v>9</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>[CSC]K410K3N</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>23.67148</v>
+      </c>
+      <c r="P14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -785,6 +940,22 @@
       <c r="J15" t="n">
         <v>7</v>
       </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>[CSC]AndMe18</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -817,6 +988,20 @@
       <c r="J16" t="n">
         <v>6</v>
       </c>
+      <c r="M16" t="n">
+        <v>11</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>[TILT]Redstony</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>23.9094</v>
+      </c>
+      <c r="P16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -849,6 +1034,20 @@
       <c r="J17" t="n">
         <v>6</v>
       </c>
+      <c r="M17" t="n">
+        <v>12</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>23.93599</v>
+      </c>
+      <c r="P17" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -879,6 +1078,22 @@
       <c r="J18" t="n">
         <v>5</v>
       </c>
+      <c r="M18" t="n">
+        <v>13</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>B_ES</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -909,6 +1124,22 @@
       <c r="J19" t="n">
         <v>5</v>
       </c>
+      <c r="M19" t="n">
+        <v>13</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>gilgool</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -941,6 +1172,20 @@
       <c r="J20" t="n">
         <v>5</v>
       </c>
+      <c r="M20" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Jorts</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>24.08418</v>
+      </c>
+      <c r="P20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -971,6 +1216,20 @@
       <c r="J21" t="n">
         <v>4</v>
       </c>
+      <c r="M21" t="n">
+        <v>16</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>[CSC] variableferret</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>24.10548</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1001,6 +1260,20 @@
       <c r="J22" t="n">
         <v>4</v>
       </c>
+      <c r="M22" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>24.61787</v>
+      </c>
+      <c r="P22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1031,6 +1304,20 @@
       <c r="J23" t="n">
         <v>4</v>
       </c>
+      <c r="M23" t="n">
+        <v>18</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>23.74024</v>
+      </c>
+      <c r="P23" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1061,6 +1348,20 @@
       <c r="J24" t="n">
         <v>4</v>
       </c>
+      <c r="M24" t="n">
+        <v>19</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>23.86045</v>
+      </c>
+      <c r="P24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1091,6 +1392,20 @@
       <c r="J25" t="n">
         <v>3</v>
       </c>
+      <c r="M25" t="n">
+        <v>20</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>23.93557</v>
+      </c>
+      <c r="P25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1123,6 +1438,20 @@
       <c r="J26" t="n">
         <v>3</v>
       </c>
+      <c r="M26" t="n">
+        <v>21</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Akane</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>24.85915</v>
+      </c>
+      <c r="P26" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1153,6 +1482,20 @@
       <c r="J27" t="n">
         <v>3</v>
       </c>
+      <c r="M27" t="n">
+        <v>22</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>25.82551</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1185,6 +1528,22 @@
       <c r="J28" t="n">
         <v>3</v>
       </c>
+      <c r="M28" t="n">
+        <v>23</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>St Nicholas</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1217,6 +1576,20 @@
       <c r="J29" t="n">
         <v>2</v>
       </c>
+      <c r="M29" t="n">
+        <v>24</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>24.40316</v>
+      </c>
+      <c r="P29" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1249,6 +1622,20 @@
       <c r="J30" t="n">
         <v>2</v>
       </c>
+      <c r="M30" t="n">
+        <v>25</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>24.52093</v>
+      </c>
+      <c r="P30" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1281,6 +1668,22 @@
       <c r="J31" t="n">
         <v>2</v>
       </c>
+      <c r="M31" t="n">
+        <v>26</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>DeiRex</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1313,6 +1716,22 @@
       <c r="J32" t="n">
         <v>2</v>
       </c>
+      <c r="M32" t="n">
+        <v>27</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Crispy</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1347,6 +1766,22 @@
       <c r="J33" t="n">
         <v>1</v>
       </c>
+      <c r="M33" t="n">
+        <v>27</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>DaimyoN</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1379,6 +1814,22 @@
         </is>
       </c>
       <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>27</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>OwenTheOmnipotent</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Petite Cup 54 (S4 Round 4): justMaki wins, first cup from the submit page
- PCDJ #53, 34 players, submitted by aizpun and processed by the poller.
- Aliases: B_ES and B_es are Vael, what_is_tatari_2008 is ZOMAN. The
  pre-cup snapshot was rebuilt with them so the arrows compare like for like.
- Poller: publish detection reads origin/master (this repo's branch).
- Tests: the guard and replay tests follow the latest cup instead of
  assuming Cup 53.
</commit_message>
<xml_diff>
--- a/Petite Cups 51-55.xlsx
+++ b/Petite Cups 51-55.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:P59"/>
+  <dimension ref="A2:V59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -432,6 +432,11 @@
           <t>Petite Cup 53</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Petite Cup 54</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -449,6 +454,11 @@
           <t>Maps: PCDJ #52 - Bankbanknewnew by [CSC] Shadynook + PCDJ #52 - A Little Bit of Bob by [CSC] redal</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #53 - rebondit by brrryy + PCDJ #53 - this map was never given a name after approval so its name is now Ger by MetalCJ</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -507,6 +517,26 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -546,6 +576,17 @@
       <c r="O6" t="n">
         <v>22.94841</v>
       </c>
+      <c r="S6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>20.56915</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -592,6 +633,22 @@
       <c r="P7" t="n">
         <v>14</v>
       </c>
+      <c r="S7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>tatari_lover2008</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -636,6 +693,20 @@
       <c r="P8" t="n">
         <v>13</v>
       </c>
+      <c r="S8" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Vael</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>18.79943</v>
+      </c>
+      <c r="V8" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -682,6 +753,20 @@
       <c r="P9" t="n">
         <v>12</v>
       </c>
+      <c r="S9" t="n">
+        <v>4</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>what_is_tatari_2008</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>20.86731</v>
+      </c>
+      <c r="V9" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -728,6 +813,20 @@
       <c r="P10" t="n">
         <v>11</v>
       </c>
+      <c r="S10" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>[WASH] Quickracer10</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>18.92304</v>
+      </c>
+      <c r="V10" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -774,6 +873,20 @@
       <c r="P11" t="n">
         <v>10</v>
       </c>
+      <c r="S11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[CSC]Tommygaming</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>21.19577</v>
+      </c>
+      <c r="V11" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -818,6 +931,20 @@
       <c r="P12" t="n">
         <v>9</v>
       </c>
+      <c r="S12" t="n">
+        <v>7</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>18.99515</v>
+      </c>
+      <c r="V12" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -862,6 +989,20 @@
       <c r="P13" t="n">
         <v>9</v>
       </c>
+      <c r="S13" t="n">
+        <v>8</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>19.17211</v>
+      </c>
+      <c r="V13" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -906,6 +1047,20 @@
       <c r="P14" t="n">
         <v>8</v>
       </c>
+      <c r="S14" t="n">
+        <v>9</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Warsnac</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>21.07061</v>
+      </c>
+      <c r="V14" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -956,6 +1111,20 @@
       <c r="P15" t="n">
         <v>8</v>
       </c>
+      <c r="S15" t="n">
+        <v>10</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Jake</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>21.15429</v>
+      </c>
+      <c r="V15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1002,6 +1171,20 @@
       <c r="P16" t="n">
         <v>7</v>
       </c>
+      <c r="S16" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>[CSC] PlusMicron</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>19.41169</v>
+      </c>
+      <c r="V16" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1048,6 +1231,20 @@
       <c r="P17" t="n">
         <v>7</v>
       </c>
+      <c r="S17" t="n">
+        <v>12</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>20.04786</v>
+      </c>
+      <c r="V17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1094,6 +1291,20 @@
       <c r="P18" t="n">
         <v>6</v>
       </c>
+      <c r="S18" t="n">
+        <v>13</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>21.12927</v>
+      </c>
+      <c r="V18" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1140,6 +1351,20 @@
       <c r="P19" t="n">
         <v>6</v>
       </c>
+      <c r="S19" t="n">
+        <v>14</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>[CSC]AndMe18</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>21.54965</v>
+      </c>
+      <c r="V19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1186,6 +1411,20 @@
       <c r="P20" t="n">
         <v>5</v>
       </c>
+      <c r="S20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>[CSC]IronDragon111000</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>19.86322</v>
+      </c>
+      <c r="V20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1230,6 +1469,22 @@
       <c r="P21" t="n">
         <v>5</v>
       </c>
+      <c r="S21" t="n">
+        <v>16</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1274,6 +1529,22 @@
       <c r="P22" t="n">
         <v>5</v>
       </c>
+      <c r="S22" t="n">
+        <v>16</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1318,6 +1589,20 @@
       <c r="P23" t="n">
         <v>4</v>
       </c>
+      <c r="S23" t="n">
+        <v>18</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>21.49061</v>
+      </c>
+      <c r="V23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1362,6 +1647,20 @@
       <c r="P24" t="n">
         <v>4</v>
       </c>
+      <c r="S24" t="n">
+        <v>19</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>21.49787</v>
+      </c>
+      <c r="V24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1406,6 +1705,22 @@
       <c r="P25" t="n">
         <v>4</v>
       </c>
+      <c r="S25" t="n">
+        <v>20</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Jorts</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1452,6 +1767,20 @@
       <c r="P26" t="n">
         <v>3</v>
       </c>
+      <c r="S26" t="n">
+        <v>21</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>wunderBarr</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>19.73848</v>
+      </c>
+      <c r="V26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1496,6 +1825,20 @@
       <c r="P27" t="n">
         <v>3</v>
       </c>
+      <c r="S27" t="n">
+        <v>22</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>19.83353</v>
+      </c>
+      <c r="V27" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1544,6 +1887,20 @@
       <c r="P28" t="n">
         <v>3</v>
       </c>
+      <c r="S28" t="n">
+        <v>23</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>M4rv</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>20.06532</v>
+      </c>
+      <c r="V28" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1590,6 +1947,20 @@
       <c r="P29" t="n">
         <v>2</v>
       </c>
+      <c r="S29" t="n">
+        <v>24</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>21.78723</v>
+      </c>
+      <c r="V29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1636,6 +2007,20 @@
       <c r="P30" t="n">
         <v>2</v>
       </c>
+      <c r="S30" t="n">
+        <v>25</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>22.33803</v>
+      </c>
+      <c r="V30" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1684,6 +2069,22 @@
       <c r="P31" t="n">
         <v>2</v>
       </c>
+      <c r="S31" t="n">
+        <v>26</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>[MMM]Kreeeeee</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1732,6 +2133,20 @@
       <c r="P32" t="n">
         <v>1</v>
       </c>
+      <c r="S32" t="n">
+        <v>27</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>20.75533</v>
+      </c>
+      <c r="V32" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1782,6 +2197,20 @@
       <c r="P33" t="n">
         <v>1</v>
       </c>
+      <c r="S33" t="n">
+        <v>28</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>VroomVroomer</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>21.29516</v>
+      </c>
+      <c r="V33" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1832,6 +2261,20 @@
       <c r="P34" t="n">
         <v>1</v>
       </c>
+      <c r="S34" t="n">
+        <v>29</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>[CSC]ShyGirlyRaccoon</t>
+        </is>
+      </c>
+      <c r="U34" t="n">
+        <v>22.17952</v>
+      </c>
+      <c r="V34" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1866,6 +2309,20 @@
       <c r="J35" t="n">
         <v>1</v>
       </c>
+      <c r="S35" t="n">
+        <v>30</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="U35" t="n">
+        <v>22.29669</v>
+      </c>
+      <c r="V35" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1900,6 +2357,20 @@
       <c r="J36" t="n">
         <v>1</v>
       </c>
+      <c r="S36" t="n">
+        <v>31</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>imagineaclevernamehere</t>
+        </is>
+      </c>
+      <c r="U36" t="n">
+        <v>22.85007</v>
+      </c>
+      <c r="V36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1934,6 +2405,20 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
+      <c r="S37" t="n">
+        <v>32</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>lele514</t>
+        </is>
+      </c>
+      <c r="U37" t="n">
+        <v>23.14757</v>
+      </c>
+      <c r="V37" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1952,6 +2437,22 @@
       <c r="D38" t="n">
         <v>1</v>
       </c>
+      <c r="S38" t="n">
+        <v>33</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>J0k3r_97</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1968,6 +2469,22 @@
         </is>
       </c>
       <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" t="n">
+        <v>33</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>LKat</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V39" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Petite Cup 55 (S4 Round 5): JakeAdjacent wins, takes the season lead
32 players, 14 elimination rounds, SOF 89.2.
Maps PCDJ #54 Deep Depths (IronDragon111000) and PCDJ #54 - Cobalt Dust
(Tommygaming). IronDragon was in the lobby and excluded as mapper;
Tommygaming was not present. The logger kept running past the final, so
the livelog holds a 15th round that timestamp correlation drops.
</commit_message>
<xml_diff>
--- a/Petite Cups 51-55.xlsx
+++ b/Petite Cups 51-55.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:V59"/>
+  <dimension ref="A2:AB59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -437,6 +437,11 @@
           <t>Petite Cup 54</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Petite Cup 55</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -459,6 +464,11 @@
           <t>Maps: PCDJ #53 - rebondit by brrryy + PCDJ #53 - this map was never given a name after approval so its name is now Ger by MetalCJ</t>
         </is>
       </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #54 Deep Depths by IronDragon111000 + PCDJ #54 - Cobalt Dust by Tommygaming</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,6 +547,26 @@
         </is>
       </c>
       <c r="V5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -587,6 +617,17 @@
       <c r="U6" t="n">
         <v>20.56915</v>
       </c>
+      <c r="Y6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Jake</t>
+        </is>
+      </c>
+      <c r="AA6" t="n">
+        <v>23.5426</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -649,6 +690,22 @@
       <c r="V7" t="n">
         <v>16</v>
       </c>
+      <c r="Y7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Kernkob</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -707,6 +764,20 @@
       <c r="V8" t="n">
         <v>15</v>
       </c>
+      <c r="Y8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>[WASH] Quickracer10</t>
+        </is>
+      </c>
+      <c r="AA8" t="n">
+        <v>21.49331</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -767,6 +838,20 @@
       <c r="V9" t="n">
         <v>14</v>
       </c>
+      <c r="Y9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>tatari_lover2008</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>23.77388</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -827,6 +912,20 @@
       <c r="V10" t="n">
         <v>13</v>
       </c>
+      <c r="Y10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>21.50312</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -887,6 +986,20 @@
       <c r="V11" t="n">
         <v>12</v>
       </c>
+      <c r="Y11" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="AA11" t="n">
+        <v>23.71815</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -945,6 +1058,20 @@
       <c r="V12" t="n">
         <v>11</v>
       </c>
+      <c r="Y12" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
+      <c r="AA12" t="n">
+        <v>23.7824</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1003,6 +1130,20 @@
       <c r="V13" t="n">
         <v>11</v>
       </c>
+      <c r="Y13" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>21.85799</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1061,6 +1202,20 @@
       <c r="V14" t="n">
         <v>10</v>
       </c>
+      <c r="Y14" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>wunderBarr</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>22.07216</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1125,6 +1280,20 @@
       <c r="V15" t="n">
         <v>10</v>
       </c>
+      <c r="Y15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>DeiRex</t>
+        </is>
+      </c>
+      <c r="AA15" t="n">
+        <v>24.16677</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1185,6 +1354,20 @@
       <c r="V16" t="n">
         <v>9</v>
       </c>
+      <c r="Y16" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="AA16" t="n">
+        <v>24.42245</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1245,6 +1428,20 @@
       <c r="V17" t="n">
         <v>9</v>
       </c>
+      <c r="Y17" t="n">
+        <v>12</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>22.13584</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1305,6 +1502,20 @@
       <c r="V18" t="n">
         <v>8</v>
       </c>
+      <c r="Y18" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>22.40115</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1365,6 +1576,20 @@
       <c r="V19" t="n">
         <v>8</v>
       </c>
+      <c r="Y19" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="AA19" t="n">
+        <v>24.34847</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1425,6 +1650,20 @@
       <c r="V20" t="n">
         <v>7</v>
       </c>
+      <c r="Y20" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>[SLOW]Zeus</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>24.5064</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1485,6 +1724,20 @@
       <c r="V21" t="n">
         <v>7</v>
       </c>
+      <c r="Y21" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>24.66253</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1545,6 +1798,20 @@
       <c r="V22" t="n">
         <v>7</v>
       </c>
+      <c r="Y22" t="n">
+        <v>17</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>[CSC]K410K3N</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>22.20403</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1603,6 +1870,20 @@
       <c r="V23" t="n">
         <v>6</v>
       </c>
+      <c r="Y23" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>[CSC] PlusMicron</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>22.20427</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1661,6 +1942,20 @@
       <c r="V24" t="n">
         <v>6</v>
       </c>
+      <c r="Y24" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>[CSC] variableferret</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>22.36437</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1721,6 +2016,20 @@
       <c r="V25" t="n">
         <v>6</v>
       </c>
+      <c r="Y25" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="AA25" t="n">
+        <v>25.00156</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1781,6 +2090,20 @@
       <c r="V26" t="n">
         <v>5</v>
       </c>
+      <c r="Y26" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Akane</t>
+        </is>
+      </c>
+      <c r="AA26" t="n">
+        <v>25.82548</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1839,6 +2162,20 @@
       <c r="V27" t="n">
         <v>5</v>
       </c>
+      <c r="Y27" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="AA27" t="n">
+        <v>27.85817</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1901,6 +2238,20 @@
       <c r="V28" t="n">
         <v>5</v>
       </c>
+      <c r="Y28" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>[CSC]ShyGirlyRaccoon</t>
+        </is>
+      </c>
+      <c r="AA28" t="n">
+        <v>24.94454</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1961,6 +2312,22 @@
       <c r="V29" t="n">
         <v>4</v>
       </c>
+      <c r="Y29" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2021,6 +2388,22 @@
       <c r="V30" t="n">
         <v>4</v>
       </c>
+      <c r="Y30" t="n">
+        <v>24</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2085,6 +2468,20 @@
       <c r="V31" t="n">
         <v>4</v>
       </c>
+      <c r="Y31" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>Timmer933</t>
+        </is>
+      </c>
+      <c r="AA31" t="n">
+        <v>25.6856</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2147,6 +2544,20 @@
       <c r="V32" t="n">
         <v>3</v>
       </c>
+      <c r="Y32" t="n">
+        <v>27</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>[bad]kkincaid97</t>
+        </is>
+      </c>
+      <c r="AA32" t="n">
+        <v>25.8501</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2211,6 +2622,20 @@
       <c r="V33" t="n">
         <v>3</v>
       </c>
+      <c r="Y33" t="n">
+        <v>28</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>LKat</t>
+        </is>
+      </c>
+      <c r="AA33" t="n">
+        <v>27.48278</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2275,6 +2700,22 @@
       <c r="V34" t="n">
         <v>3</v>
       </c>
+      <c r="Y34" t="n">
+        <v>29</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Hellmet</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2323,6 +2764,22 @@
       <c r="V35" t="n">
         <v>2</v>
       </c>
+      <c r="Y35" t="n">
+        <v>29</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2371,6 +2828,22 @@
       <c r="V36" t="n">
         <v>2</v>
       </c>
+      <c r="Y36" t="n">
+        <v>29</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>[CSC]AndMe18</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2418,6 +2891,22 @@
       </c>
       <c r="V37" t="n">
         <v>2</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>29</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>cookie</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">

</xml_diff>